<commit_message>
fix(tienda-en): revisión final del Gastro Pro Prompts eBook — afirmaciones veraces, cheat sheet, maqueta y nombres
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/ai-prompts-for-restaurants/bonus-2-3-templates-cheat-sheet.xlsx
+++ b/astro-site/public/dl/ai-prompts-for-restaurants/bonus-2-3-templates-cheat-sheet.xlsx
@@ -824,7 +824,7 @@
           <t>Act as an executive chef specializing in [CUISINE TYPE]. Create a [LEVEL] recipe featuring [MAIN INGREDIENT] as the star.
 Context: my restaurant is [BRIEF RESTAURANT DESCRIPTION], average check [AVERAGE CHECK $], [N SEATS] seats.
 The recipe must: use [MAIN TECHNIQUE], be ready in [PREP TIME], respect the [SEASON] season, avoid [ALLERGENS TO AVOID].
-Format: dish name, story (2 sentences), ingredients with weights for [N SERVINGS] servings, step-by-step method, plating, pairing.</t>
+Format: dish name, story (2 sentences), ingredients with weights for [N SERVINGS], step-by-step method, plating, pairing.</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Kitchen · ChatGPT · Claude · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Kitchen · Works with: ChatGPT · Claude · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
 Target selling price: [SELLING PRICE $]
 Prep time: [PREP MINUTES]
 Labor cost per hour: [LABOR COST PER HOUR $]
-I need: cost table by ingredient, total ingredient cost, labor cost, gross margin, food cost %, and a menu price recommendation if the food cost exceeds [MAX FOOD COST %]%.</t>
+I need: cost table by ingredient, total ingredient cost, labor cost, gross margin, food cost %, and a menu price recommendation if the food cost exceeds [MAX FOOD COST %].</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Costing · ChatGPT · Gemini · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Costing · Works with: ChatGPT · Gemini · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Costing · Claude · ChatGPT · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Costing · Works with: Claude · ChatGPT · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Catering · ChatGPT · Claude · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Catering · Works with: ChatGPT · Claude · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Marketing · ChatGPT · Claude · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Marketing · Works with: ChatGPT · Claude · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Marketing · Claude · ChatGPT · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Marketing · Works with: Claude · ChatGPT · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Deep Research · Perplexity · Claude · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Deep Research · Works with: Perplexity · Claude · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Marketing · ChatGPT · Claude · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Marketing · Works with: ChatGPT · Claude · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Deep Research · Claude · ChatGPT · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Deep Research · Works with: Claude · ChatGPT · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Works with: Leadership · Claude · ChatGPT · AI Chef Pro</t>
+          <t xml:space="preserve">  Category: Leadership · Works with: Claude · ChatGPT · AI Chef Pro</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quick reference for everyday use. Look up the prompt number in the eBook or in AI Chef Pro to see the full prompt.</t>
+          <t>Quick reference for everyday use. Look up the number in your online dashboard (Prompt Library) to see the full prompt.</t>
         </is>
       </c>
     </row>
@@ -2438,22 +2438,22 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>#77</t>
+          <t>Bonus 1</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Master prompt generator</t>
+          <t>Build your own prompts</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>To create your own prompts</t>
+          <t>When no template fits: use the 5-element method in Bonus 1</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
         <is>
-          <t>AI Chef Pro · Claude · ChatGPT</t>
+          <t>AI Chef Pro · ChatGPT · Claude</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4.  Putting the role at the start of the prompt improves quality by up to 40%.</t>
+          <t xml:space="preserve">  4.  Putting the role first noticeably improves the answer.</t>
         </is>
       </c>
       <c r="B29" s="27" t="n"/>

</xml_diff>